<commit_message>
Swap step 1 (Vendor) and step 2 (Category)
</commit_message>
<xml_diff>
--- a/Hia_Solar_Drawing_Portal_Automation_v2.xlsx
+++ b/Hia_Solar_Drawing_Portal_Automation_v2.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="10440" activeTab="2"/>
+    <workbookView windowWidth="22188" windowHeight="10440" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="HTML Generator Dashboard" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Drawing List Database'!$A$1:$F$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$B$2:$E$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$B$2:$E$86</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="376">
   <si>
     <t>Hia Solar Master Design v2.0 - LINE OA Drawing Content Portal Generator</t>
   </si>
@@ -470,6 +470,15 @@
     <t>New request-11</t>
   </si>
   <si>
+    <t>2-Layer</t>
+  </si>
+  <si>
+    <t>E1-T2-MRV-3+3PV-4+2PV</t>
+  </si>
+  <si>
+    <t>wait</t>
+  </si>
+  <si>
     <t>Structure Name</t>
   </si>
   <si>
@@ -1149,6 +1158,9 @@
   </si>
   <si>
     <t>1TrCr793kbOCo5707Pxb0TYkYrBuWIGo3</t>
+  </si>
+  <si>
+    <t>E1-T2-MRV-3+3PV-4+2PVใยกด</t>
   </si>
 </sst>
 </file>
@@ -1161,14 +1173,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="32">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1395,7 +1400,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1585,12 +1590,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1896,137 +1895,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2034,65 +2033,68 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2200,7 +2202,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Slicer Style 1 2" pivot="0" table="0" count="7" xr9:uid="{CB9738D4-A4D3-49BC-BA9B-09333C9117AB}">
+    <tableStyle name="Slicer Style 1 2" pivot="0" table="0" count="7" xr9:uid="{383CB8D0-B64E-4D79-82DD-1E26D023333B}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -2597,12 +2599,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="24.6" spans="1:1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" ht="15" spans="1:1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2615,7 +2617,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="29.8981481481481" customWidth="1"/>
@@ -4411,6 +4413,23 @@
         <v>1D0fPzrHWduR11PsbIv2Bw0xtQNsKDbNH</v>
       </c>
     </row>
+    <row r="86" ht="15.15" spans="1:6">
+      <c r="A86" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B86" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C86" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="D86" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="E86" s="22" t="s">
+        <v>147</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F85" etc:filterBottomFollowUsedRange="0">
     <extLst/>
@@ -4423,7 +4442,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="B1:F85"/>
+  <dimension ref="B1:F86"/>
   <sheetFormatPr defaultColWidth="8.89814814814815" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="8.89814814814815" style="1"/>
@@ -4438,21 +4457,21 @@
     <row r="1" ht="15.15"/>
     <row r="2" ht="15.15" spans="2:6">
       <c r="B2" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" ht="15.15" spans="2:6">
       <c r="B3" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>126</v>
@@ -4461,7 +4480,7 @@
         <v>123456789</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F3" s="1" t="str">
         <f>_xlfn.XLOOKUP(C3,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4470,16 +4489,16 @@
     </row>
     <row r="4" ht="15.15" spans="2:6">
       <c r="B4" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F4" s="1" t="str">
         <f>_xlfn.XLOOKUP(C4,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4488,16 +4507,16 @@
     </row>
     <row r="5" ht="15.15" spans="2:6">
       <c r="B5" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F5" s="1" t="str">
         <f>_xlfn.XLOOKUP(C5,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4506,7 +4525,7 @@
     </row>
     <row r="6" ht="15.15" spans="2:6">
       <c r="B6" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>47</v>
@@ -4515,7 +4534,7 @@
         <v>48</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F6" s="1" t="str">
         <f>_xlfn.XLOOKUP(C6,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4524,7 +4543,7 @@
     </row>
     <row r="7" ht="15.15" spans="2:6">
       <c r="B7" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>34</v>
@@ -4533,7 +4552,7 @@
         <v>81301500165</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F7" s="1" t="str">
         <f>_xlfn.XLOOKUP(C7,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4542,7 +4561,7 @@
     </row>
     <row r="8" ht="15.15" spans="2:6">
       <c r="B8" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>139</v>
@@ -4551,7 +4570,7 @@
         <v>140</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F8" s="1" t="str">
         <f>_xlfn.XLOOKUP(C8,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4560,7 +4579,7 @@
     </row>
     <row r="9" ht="15.15" spans="2:6">
       <c r="B9" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>26</v>
@@ -4569,7 +4588,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F9" s="1" t="str">
         <f>_xlfn.XLOOKUP(C9,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4578,7 +4597,7 @@
     </row>
     <row r="10" ht="15.15" spans="2:6">
       <c r="B10" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>24</v>
@@ -4587,7 +4606,7 @@
         <v>25</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F10" s="1" t="str">
         <f>_xlfn.XLOOKUP(C10,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4596,7 +4615,7 @@
     </row>
     <row r="11" ht="15.15" spans="2:6">
       <c r="B11" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>22</v>
@@ -4605,7 +4624,7 @@
         <v>23</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F11" s="1" t="str">
         <f>_xlfn.XLOOKUP(C11,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4614,7 +4633,7 @@
     </row>
     <row r="12" ht="15.15" spans="2:6">
       <c r="B12" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>20</v>
@@ -4623,7 +4642,7 @@
         <v>21</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F12" s="1" t="str">
         <f>_xlfn.XLOOKUP(C12,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4632,7 +4651,7 @@
     </row>
     <row r="13" ht="15.15" spans="2:6">
       <c r="B13" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>143</v>
@@ -4641,7 +4660,7 @@
         <v>144</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F13" s="1" t="str">
         <f>_xlfn.XLOOKUP(C13,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4650,16 +4669,16 @@
     </row>
     <row r="14" ht="15.15" spans="2:6">
       <c r="B14" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F14" s="1" t="str">
         <f>_xlfn.XLOOKUP(C14,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4668,16 +4687,16 @@
     </row>
     <row r="15" ht="15.15" spans="2:6">
       <c r="B15" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>31</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F15" s="1" t="str">
         <f>_xlfn.XLOOKUP(C15,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4686,16 +4705,16 @@
     </row>
     <row r="16" ht="15.15" spans="2:6">
       <c r="B16" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>53</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F16" s="1" t="str">
         <f>_xlfn.XLOOKUP(C16,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4704,7 +4723,7 @@
     </row>
     <row r="17" ht="15.15" spans="2:6">
       <c r="B17" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>121</v>
@@ -4713,7 +4732,7 @@
         <v>81301500245</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F17" s="1" t="str">
         <f>_xlfn.XLOOKUP(C17,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4722,7 +4741,7 @@
     </row>
     <row r="18" ht="15.15" spans="2:6">
       <c r="B18" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>11</v>
@@ -4731,7 +4750,7 @@
         <v>81301500168</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F18" s="1" t="str">
         <f>_xlfn.XLOOKUP(C18,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4740,16 +4759,16 @@
     </row>
     <row r="19" ht="15.15" spans="2:6">
       <c r="B19" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>110</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F19" s="1" t="str">
         <f>_xlfn.XLOOKUP(C19,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4758,16 +4777,16 @@
     </row>
     <row r="20" ht="15.15" spans="2:6">
       <c r="B20" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>101</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F20" s="1" t="str">
         <f>_xlfn.XLOOKUP(C20,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4776,16 +4795,16 @@
     </row>
     <row r="21" ht="15.15" spans="2:6">
       <c r="B21" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F21" s="1" t="str">
         <f>_xlfn.XLOOKUP(C21,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4794,16 +4813,16 @@
     </row>
     <row r="22" ht="15.15" spans="2:6">
       <c r="B22" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>37</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F22" s="1" t="str">
         <f>_xlfn.XLOOKUP(C22,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4812,7 +4831,7 @@
     </row>
     <row r="23" ht="15.15" spans="2:6">
       <c r="B23" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>136</v>
@@ -4821,7 +4840,7 @@
         <v>81301500172</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F23" s="1" t="str">
         <f>_xlfn.XLOOKUP(C23,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4830,7 +4849,7 @@
     </row>
     <row r="24" ht="15.15" spans="2:6">
       <c r="B24" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>135</v>
@@ -4839,7 +4858,7 @@
         <v>81301500170</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F24" s="1" t="str">
         <f>_xlfn.XLOOKUP(C24,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4848,16 +4867,16 @@
     </row>
     <row r="25" ht="15.15" spans="2:6">
       <c r="B25" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>133</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F25" s="1" t="str">
         <f>_xlfn.XLOOKUP(C25,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4866,16 +4885,16 @@
     </row>
     <row r="26" ht="15.15" spans="2:6">
       <c r="B26" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>127</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F26" s="1" t="str">
         <f>_xlfn.XLOOKUP(C26,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4884,7 +4903,7 @@
     </row>
     <row r="27" ht="15.15" spans="2:6">
       <c r="B27" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>122</v>
@@ -4893,7 +4912,7 @@
         <v>81301500250</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F27" s="1" t="str">
         <f>_xlfn.XLOOKUP(C27,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4902,16 +4921,16 @@
     </row>
     <row r="28" ht="15.15" spans="2:6">
       <c r="B28" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>81</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F28" s="1" t="str">
         <f>_xlfn.XLOOKUP(C28,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4920,16 +4939,16 @@
     </row>
     <row r="29" ht="15.15" spans="2:6">
       <c r="B29" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>74</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F29" s="1" t="str">
         <f>_xlfn.XLOOKUP(C29,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4938,16 +4957,16 @@
     </row>
     <row r="30" ht="15.15" spans="2:6">
       <c r="B30" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>72</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F30" s="1" t="str">
         <f>_xlfn.XLOOKUP(C30,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4956,16 +4975,16 @@
     </row>
     <row r="31" ht="15.15" spans="2:6">
       <c r="B31" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F31" s="1" t="str">
         <f>_xlfn.XLOOKUP(C31,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4974,16 +4993,16 @@
     </row>
     <row r="32" ht="15.15" spans="2:6">
       <c r="B32" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>54</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F32" s="1" t="str">
         <f>_xlfn.XLOOKUP(C32,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -4992,7 +5011,7 @@
     </row>
     <row r="33" ht="15.15" spans="2:6">
       <c r="B33" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>39</v>
@@ -5001,7 +5020,7 @@
         <v>81301500244</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F33" s="1" t="str">
         <f>_xlfn.XLOOKUP(C33,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5010,16 +5029,16 @@
     </row>
     <row r="34" ht="15.15" spans="2:6">
       <c r="B34" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>29</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F34" s="1" t="str">
         <f>_xlfn.XLOOKUP(C34,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5028,16 +5047,16 @@
     </row>
     <row r="35" ht="15.15" spans="2:6">
       <c r="B35" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F35" s="1" t="str">
         <f>_xlfn.XLOOKUP(C35,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5046,7 +5065,7 @@
     </row>
     <row r="36" ht="15.15" spans="2:6">
       <c r="B36" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>15</v>
@@ -5055,7 +5074,7 @@
         <v>81301500257</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F36" s="1" t="str">
         <f>_xlfn.XLOOKUP(C36,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5064,16 +5083,16 @@
     </row>
     <row r="37" ht="15.15" spans="2:6">
       <c r="B37" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>131</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F37" s="1" t="str">
         <f>_xlfn.XLOOKUP(C37,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5082,16 +5101,16 @@
     </row>
     <row r="38" ht="15.15" spans="2:6">
       <c r="B38" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>130</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F38" s="1" t="str">
         <f>_xlfn.XLOOKUP(C38,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5100,16 +5119,16 @@
     </row>
     <row r="39" ht="15.15" spans="2:6">
       <c r="B39" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>129</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F39" s="1" t="str">
         <f>_xlfn.XLOOKUP(C39,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5118,16 +5137,16 @@
     </row>
     <row r="40" ht="15.15" spans="2:6">
       <c r="B40" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>128</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F40" s="1" t="str">
         <f>_xlfn.XLOOKUP(C40,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5136,7 +5155,7 @@
     </row>
     <row r="41" ht="15.15" spans="2:6">
       <c r="B41" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>137</v>
@@ -5145,7 +5164,7 @@
         <v>138</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F41" s="1" t="str">
         <f>_xlfn.XLOOKUP(C41,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5154,7 +5173,7 @@
     </row>
     <row r="42" ht="15.15" spans="2:6">
       <c r="B42" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>141</v>
@@ -5163,7 +5182,7 @@
         <v>142</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="F42" s="1" t="str">
         <f>_xlfn.XLOOKUP(C42,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5172,16 +5191,16 @@
     </row>
     <row r="43" ht="15.15" spans="2:6">
       <c r="B43" s="3" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D43" s="5">
         <v>0</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F43" s="1">
         <f>_xlfn.XLOOKUP(C43,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5190,16 +5209,16 @@
     </row>
     <row r="44" ht="15.15" spans="2:6">
       <c r="B44" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F44" s="1" t="str">
         <f>_xlfn.XLOOKUP(C44,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5208,7 +5227,7 @@
     </row>
     <row r="45" ht="15.15" spans="2:6">
       <c r="B45" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>115</v>
@@ -5217,7 +5236,7 @@
         <v>116</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F45" s="1" t="str">
         <f>_xlfn.XLOOKUP(C45,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5226,16 +5245,16 @@
     </row>
     <row r="46" ht="15.15" spans="2:6">
       <c r="B46" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>119</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F46" s="1" t="str">
         <f>_xlfn.XLOOKUP(C46,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5244,7 +5263,7 @@
     </row>
     <row r="47" ht="15.15" spans="2:6">
       <c r="B47" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>117</v>
@@ -5253,7 +5272,7 @@
         <v>118</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F47" s="1" t="str">
         <f>_xlfn.XLOOKUP(C47,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5262,7 +5281,7 @@
     </row>
     <row r="48" ht="15.15" spans="2:6">
       <c r="B48" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>33</v>
@@ -5271,7 +5290,7 @@
         <v>81301500262</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F48" s="1" t="str">
         <f>_xlfn.XLOOKUP(C48,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5280,7 +5299,7 @@
     </row>
     <row r="49" ht="15.15" spans="2:6">
       <c r="B49" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>76</v>
@@ -5289,7 +5308,7 @@
         <v>0</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F49" s="1" t="str">
         <f>_xlfn.XLOOKUP(C49,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5298,7 +5317,7 @@
     </row>
     <row r="50" ht="15.15" spans="2:6">
       <c r="B50" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>75</v>
@@ -5307,7 +5326,7 @@
         <v>0</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F50" s="1" t="str">
         <f>_xlfn.XLOOKUP(C50,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5316,16 +5335,16 @@
     </row>
     <row r="51" ht="15.15" spans="2:6">
       <c r="B51" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F51" s="1" t="str">
         <f>_xlfn.XLOOKUP(C51,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5334,7 +5353,7 @@
     </row>
     <row r="52" ht="15.15" spans="2:6">
       <c r="B52" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>13</v>
@@ -5343,7 +5362,7 @@
         <v>81301500160</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F52" s="1" t="str">
         <f>_xlfn.XLOOKUP(C52,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5352,16 +5371,16 @@
     </row>
     <row r="53" ht="15.15" spans="2:6">
       <c r="B53" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="F53" s="1" t="str">
         <f>_xlfn.XLOOKUP(C53,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5370,7 +5389,7 @@
     </row>
     <row r="54" ht="15.15" spans="2:6">
       <c r="B54" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>44</v>
@@ -5379,7 +5398,7 @@
         <v>45</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="F54" s="1" t="str">
         <f>_xlfn.XLOOKUP(C54,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5388,16 +5407,16 @@
     </row>
     <row r="55" ht="15.15" spans="2:6">
       <c r="B55" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>113</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F55" s="1" t="str">
         <f>_xlfn.XLOOKUP(C55,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5406,16 +5425,16 @@
     </row>
     <row r="56" ht="15.15" spans="2:6">
       <c r="B56" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F56" s="1" t="str">
         <f>_xlfn.XLOOKUP(C56,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5424,16 +5443,16 @@
     </row>
     <row r="57" ht="15.15" spans="2:6">
       <c r="B57" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>111</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F57" s="1" t="str">
         <f>_xlfn.XLOOKUP(C57,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5442,16 +5461,16 @@
     </row>
     <row r="58" ht="15.15" spans="2:6">
       <c r="B58" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>106</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F58" s="1" t="str">
         <f>_xlfn.XLOOKUP(C58,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5460,16 +5479,16 @@
     </row>
     <row r="59" ht="15.15" spans="2:6">
       <c r="B59" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>105</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F59" s="1" t="str">
         <f>_xlfn.XLOOKUP(C59,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5478,16 +5497,16 @@
     </row>
     <row r="60" ht="15.15" spans="2:6">
       <c r="B60" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>100</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F60" s="1" t="str">
         <f>_xlfn.XLOOKUP(C60,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5496,16 +5515,16 @@
     </row>
     <row r="61" ht="15.15" spans="2:6">
       <c r="B61" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>97</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F61" s="1" t="str">
         <f>_xlfn.XLOOKUP(C61,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5514,16 +5533,16 @@
     </row>
     <row r="62" ht="15.15" spans="2:6">
       <c r="B62" s="2" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F62" s="1" t="str">
         <f>_xlfn.XLOOKUP(C62,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5532,16 +5551,16 @@
     </row>
     <row r="63" ht="15.15" spans="2:6">
       <c r="B63" s="2" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>102</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F63" s="1" t="str">
         <f>_xlfn.XLOOKUP(C63,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5550,16 +5569,16 @@
     </row>
     <row r="64" ht="15.15" spans="2:6">
       <c r="B64" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>109</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="F64" s="1" t="str">
         <f>_xlfn.XLOOKUP(C64,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5568,16 +5587,16 @@
     </row>
     <row r="65" ht="15.15" spans="2:6">
       <c r="B65" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>91</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F65" s="1" t="str">
         <f>_xlfn.XLOOKUP(C65,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5586,16 +5605,16 @@
     </row>
     <row r="66" ht="15.15" spans="2:6">
       <c r="B66" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>89</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F66" s="1" t="str">
         <f>_xlfn.XLOOKUP(C66,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5604,16 +5623,16 @@
     </row>
     <row r="67" ht="15.15" spans="2:6">
       <c r="B67" s="2" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F67" s="1" t="str">
         <f>_xlfn.XLOOKUP(C67,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5622,16 +5641,16 @@
     </row>
     <row r="68" ht="15.15" spans="2:6">
       <c r="B68" s="2" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>88</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F68" s="1" t="str">
         <f>_xlfn.XLOOKUP(C68,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5640,16 +5659,16 @@
     </row>
     <row r="69" ht="15.15" spans="2:6">
       <c r="B69" s="2" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>87</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F69" s="1" t="str">
         <f>_xlfn.XLOOKUP(C69,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5658,16 +5677,16 @@
     </row>
     <row r="70" ht="15.15" spans="2:6">
       <c r="B70" s="2" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>85</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F70" s="1" t="str">
         <f>_xlfn.XLOOKUP(C70,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5676,16 +5695,16 @@
     </row>
     <row r="71" ht="15.15" spans="2:6">
       <c r="B71" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>80</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F71" s="1" t="str">
         <f>_xlfn.XLOOKUP(C71,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5694,16 +5713,16 @@
     </row>
     <row r="72" ht="15.15" spans="2:6">
       <c r="B72" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>83</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F72" s="1" t="str">
         <f>_xlfn.XLOOKUP(C72,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5712,16 +5731,16 @@
     </row>
     <row r="73" ht="15.15" spans="2:6">
       <c r="B73" s="2" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>78</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F73" s="1" t="str">
         <f>_xlfn.XLOOKUP(C73,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5730,16 +5749,16 @@
     </row>
     <row r="74" ht="15.15" spans="2:6">
       <c r="B74" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>77</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F74" s="1" t="str">
         <f>_xlfn.XLOOKUP(C74,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5748,16 +5767,16 @@
     </row>
     <row r="75" ht="15.15" spans="2:6">
       <c r="B75" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>70</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F75" s="1" t="str">
         <f>_xlfn.XLOOKUP(C75,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5766,16 +5785,16 @@
     </row>
     <row r="76" ht="15.15" spans="2:6">
       <c r="B76" s="2" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>69</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F76" s="1" t="str">
         <f>_xlfn.XLOOKUP(C76,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5784,16 +5803,16 @@
     </row>
     <row r="77" ht="15.15" spans="2:6">
       <c r="B77" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>132</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F77" s="1" t="str">
         <f>_xlfn.XLOOKUP(C77,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5802,16 +5821,16 @@
     </row>
     <row r="78" ht="15.15" spans="2:6">
       <c r="B78" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="F78" s="1" t="str">
         <f>_xlfn.XLOOKUP(C78,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5820,16 +5839,16 @@
     </row>
     <row r="79" ht="15.15" spans="2:6">
       <c r="B79" s="2" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>67</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F79" s="1" t="str">
         <f>_xlfn.XLOOKUP(C79,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5838,16 +5857,16 @@
     </row>
     <row r="80" ht="15.15" spans="2:6">
       <c r="B80" s="2" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="F80" s="1" t="str">
         <f>_xlfn.XLOOKUP(C80,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5856,16 +5875,16 @@
     </row>
     <row r="81" ht="15.15" spans="2:6">
       <c r="B81" s="2" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>64</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="F81" s="1" t="str">
         <f>_xlfn.XLOOKUP(C81,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5874,16 +5893,16 @@
     </row>
     <row r="82" ht="15.15" spans="2:6">
       <c r="B82" s="2" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>62</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="F82" s="1" t="str">
         <f>_xlfn.XLOOKUP(C82,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5892,16 +5911,16 @@
     </row>
     <row r="83" ht="15.15" spans="2:6">
       <c r="B83" s="2" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>61</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="F83" s="1" t="str">
         <f>_xlfn.XLOOKUP(C83,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5910,16 +5929,16 @@
     </row>
     <row r="84" ht="15.15" spans="2:6">
       <c r="B84" s="2" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="F84" s="1" t="str">
         <f>_xlfn.XLOOKUP(C84,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
@@ -5928,24 +5947,38 @@
     </row>
     <row r="85" ht="15.15" spans="2:6">
       <c r="B85" s="2" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="F85" s="1" t="str">
         <f>_xlfn.XLOOKUP(C85,'Drawing List Database'!D:D,'Drawing List Database'!B:B,0)</f>
         <v>TCC</v>
       </c>
     </row>
+    <row r="86" spans="2:6">
+      <c r="B86" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:E85" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:E86" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>